<commit_message>
version beta 2 - semaine 3
</commit_message>
<xml_diff>
--- a/template/horaire.xlsx
+++ b/template/horaire.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/etiennerivard/notes_de_cours/web3/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{454760B1-C5EF-DC45-9352-261612B09E09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D8D34B2-5E2C-C346-A9F6-4A7443C01CEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3000" yWindow="1580" windowWidth="25920" windowHeight="16440" xr2:uid="{4696F4E7-E751-AB46-8D30-A385E7EE1466}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="47">
   <si>
     <t>Date</t>
   </si>
@@ -56,61 +56,127 @@
     <t>Examen React</t>
   </si>
   <si>
-    <t>[lodash](exercices/lodash.md)</t>
-  </si>
-  <si>
     <t>Retour sur formatif &lt;br/&gt; Période de questions</t>
   </si>
   <si>
     <t>[Introduction à Next.js](lecons/next.js/introduction.md)</t>
   </si>
   <si>
-    <t>Projet Intégrateur</t>
-  </si>
-  <si>
-    <t>Projet Intégrateur (remise à la fin du cours)</t>
-  </si>
-  <si>
-    <t>[Introduction React](exercices/react_intro.md)</t>
-  </si>
-  <si>
-    <t>[React et les styles](exercices/react_styles.md)</t>
-  </si>
-  <si>
-    <t>[React et les routes](exercices/react_routes.md)</t>
-  </si>
-  <si>
-    <t>[React et contexte](exercices/react_contexte.md)</t>
-  </si>
-  <si>
-    <t>[React et l'Internatialisation](exercices/internationalisation.md)</t>
-  </si>
-  <si>
     <t xml:space="preserve">[Introduction à TypeScript](lecons/typescript/introduction_typescript.md) &lt;br/&gt; [npm](lecons/typescript/npm.md) &lt;br/&gt;[Prettier](lecons/typescript/prettier.md)  </t>
   </si>
   <si>
     <t>[TypeScript 2](lecons/typescript/typescript_2.md)&lt;br/&gt;[JavaScript asynchrone](lecons/typescript/javascript_async.md)</t>
   </si>
   <si>
-    <t>[Introduction à React](lecons/react/introduction_react.md)&lt;br/&gt; [Structure typique d'un projet React](lecons/react/structure_projet_react.md)&lt;br/&gt; [Penser en React](lecons/react/penser_en_react.md)</t>
-  </si>
-  <si>
-    <t>[Styles : React et MUI](lecons/react/react_mui.md)&lt;br/&gt; [Styles : TailWindCSS](lecons/react/react_tw.md)</t>
-  </si>
-  <si>
     <t>[Routes](lecons/react/react3.md)</t>
   </si>
   <si>
-    <t>[Contexte et API](lecons/react/react4.md)&lt;br/&gt; [Régles de React](lecons/react/regles_react.md)</t>
-  </si>
-  <si>
     <t>[Internationalisation](lecons/react/internationalisation.md)</t>
   </si>
   <si>
     <t>[React dans Azure](lecons/deploiement/azure_react.md)</t>
   </si>
   <si>
-    <t>[Azure](exercices/azure.md)</t>
+    <t>[Introduction à React](lecons/react/introduction_react.md)&lt;br/&gt; [Structure typique d'un projet React](lecons/react/structure_projet_react.md)&lt;br/&gt; [useState](lecons/react/react_usestate.md) &lt;br/&gt; [useEffect](lecons/react/react_useeffect.md)</t>
+  </si>
+  <si>
+    <t>[Styles : TailWindCSS](lecons/react/react_tw.md) &lt;br/&gt; [shadcn/UI](lecons/react/react_shadcn)</t>
+  </si>
+  <si>
+    <t>[Penser en React](lecons/react/penser_en_react.md) &lt;br/&gt; [Mécanique de React](lecons/react/mecanique_react.md)</t>
+  </si>
+  <si>
+    <t>Projet formatif next.js</t>
+  </si>
+  <si>
+    <t>Pratique d'examen final</t>
+  </si>
+  <si>
+    <t>Retour sur pratique d'examen final</t>
+  </si>
+  <si>
+    <t>[Routage dans Next.js](lecons/next.js/routage.md)</t>
+  </si>
+  <si>
+    <t>[Modes de rendu](lecons/next.js/modes_rendu.md)</t>
+  </si>
+  <si>
+    <t>[Routes API](lecons/next.js/api_routes.md)</t>
+  </si>
+  <si>
+    <t>[Server Actions et formulaires](lecons/next.js/server_actions.md)</t>
+  </si>
+  <si>
+    <t>[Immer](lecons/outils/immer.md)</t>
+  </si>
+  <si>
+    <t>[useReducer](lecons/react/react_usereducer.md)</t>
+  </si>
+  <si>
+    <t>[Prisma ORM](lecons/next.js/orm.md)</t>
+  </si>
+  <si>
+    <t>[API](lecons/react/react4.md)&lt;br/&gt; [useContext](lecons/react/react_usecontext.md)&lt;br/&gt; [Règles de React](lecons/react/regles_react.md)</t>
+  </si>
+  <si>
+    <t>[Internationalisation avec Next.js](lecons/next.js/next_intl.md)</t>
+  </si>
+  <si>
+    <t>[Intro à Next.js](exercices/next_intro.md)</t>
+  </si>
+  <si>
+    <t>[Routage dans Next.js](exercices/next_routage.md)</t>
+  </si>
+  <si>
+    <t>[Composantes dans Next.js](exercices/next_composantes.md)</t>
+  </si>
+  <si>
+    <t>[Modes de rendu](exercices/next_modes_rendu.md)</t>
+  </si>
+  <si>
+    <t>[Hydratation](lecons/next.js/hydratation.md)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Composantes serveur VS client](lecons/next.js/composantes.md) </t>
+  </si>
+  <si>
+    <t>[Hydratation](exercices/next_hydratation.md)</t>
+  </si>
+  <si>
+    <t>[Routes API](exercices/next_api_routes.md)</t>
+  </si>
+  <si>
+    <t>[ORM](exercices/next_orm.md)</t>
+  </si>
+  <si>
+    <t>[Server Actions](exercices/next_server_actions.md)</t>
+  </si>
+  <si>
+    <t>[Internationalisation](exercices/next_intl_exercice.md)</t>
+  </si>
+  <si>
+    <t>[Introduction React](exercices/react/react_intro.md)</t>
+  </si>
+  <si>
+    <t>[Penser en React et Mécanique de React](exercices/react/react_penser_mecanique.md)</t>
+  </si>
+  <si>
+    <t>[React et les styles](exercices/react/react_styles.md)</t>
+  </si>
+  <si>
+    <t>[React et les routes](exercices/react/react_routes.md)</t>
+  </si>
+  <si>
+    <t>[React et contexte](exercices/react/react_contexte.md)</t>
+  </si>
+  <si>
+    <t>[React et l'Internationalisation](exercices/react/react_intl.md)</t>
+  </si>
+  <si>
+    <t>[lodash](exercices/typescript/lodash.md)</t>
+  </si>
+  <si>
+    <t>[Typescript 2 et JavaScript asynchrone](exercices/typescript/typescript_async.md)</t>
   </si>
 </sst>
 </file>
@@ -509,7 +575,8 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="142.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="103.33203125" customWidth="1"/>
+    <col min="4" max="4" width="66" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
@@ -531,13 +598,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="1">
-        <v>45890.552083333336</v>
+        <v>46254.427083333336</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -545,10 +612,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="2">
-        <v>45894.510416666664</v>
+        <v>46259.59375</v>
       </c>
       <c r="C3" t="s">
-        <v>17</v>
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -556,13 +626,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="1">
-        <v>45897.552083333336</v>
+        <v>46261.427083333336</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="D4" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -570,13 +640,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="2">
-        <v>45904.510416666664</v>
+        <v>46268.427083333336</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D5" t="s">
-        <v>12</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -584,13 +654,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="1">
-        <v>45908.510416666664</v>
+        <v>46273.59375</v>
       </c>
       <c r="C6" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="D6" t="s">
-        <v>13</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -598,13 +668,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="2">
-        <v>45911.552083333336</v>
+        <v>46276.59375</v>
       </c>
       <c r="C7" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="D7" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -612,13 +682,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="1">
-        <v>45915.510416666664</v>
+        <v>46280.59375</v>
       </c>
       <c r="C8" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D8" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -626,10 +696,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="2">
-        <v>45918.552083333336</v>
+        <v>46282.427083333336</v>
       </c>
       <c r="C9" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
@@ -637,10 +707,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="1">
-        <v>45922.510416666664</v>
+        <v>46287.59375</v>
       </c>
       <c r="C10" t="s">
-        <v>7</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
@@ -648,10 +718,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="2">
-        <v>45925.552083333336</v>
+        <v>46289.427083333336</v>
       </c>
       <c r="C11" t="s">
-        <v>8</v>
+        <v>11</v>
+      </c>
+      <c r="D11" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
@@ -659,10 +732,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="1">
-        <v>45929.510416666664</v>
+        <v>46294.59375</v>
       </c>
       <c r="C12" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
@@ -670,7 +743,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="2">
-        <v>45932.552083333336</v>
+        <v>46296.427083333336</v>
+      </c>
+      <c r="C13" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
@@ -678,7 +754,13 @@
         <v>13</v>
       </c>
       <c r="B14" s="1">
-        <v>45936.510416666664</v>
+        <v>46301.59375</v>
+      </c>
+      <c r="C14" t="s">
+        <v>7</v>
+      </c>
+      <c r="D14" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
@@ -686,7 +768,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="2">
-        <v>45939.552083333336</v>
+        <v>46303.427083333336</v>
+      </c>
+      <c r="C15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
@@ -694,7 +779,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="1">
-        <v>45950.510416666664</v>
+        <v>46315.59375</v>
+      </c>
+      <c r="C16" t="s">
+        <v>19</v>
+      </c>
+      <c r="D16" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
@@ -702,7 +793,13 @@
         <v>16</v>
       </c>
       <c r="B17" s="2">
-        <v>45953.552083333336</v>
+        <v>46317.427083333336</v>
+      </c>
+      <c r="C17" t="s">
+        <v>33</v>
+      </c>
+      <c r="D17" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
@@ -710,7 +807,13 @@
         <v>17</v>
       </c>
       <c r="B18" s="1">
-        <v>45957.510416666664</v>
+        <v>46322.59375</v>
+      </c>
+      <c r="C18" t="s">
+        <v>20</v>
+      </c>
+      <c r="D18" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
@@ -718,7 +821,13 @@
         <v>18</v>
       </c>
       <c r="B19" s="2">
-        <v>45960.552083333336</v>
+        <v>46324.427083333336</v>
+      </c>
+      <c r="C19" t="s">
+        <v>32</v>
+      </c>
+      <c r="D19" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
@@ -726,7 +835,13 @@
         <v>19</v>
       </c>
       <c r="B20" s="1">
-        <v>45967.552083333336</v>
+        <v>46329.59375</v>
+      </c>
+      <c r="C20" t="s">
+        <v>21</v>
+      </c>
+      <c r="D20" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
@@ -734,7 +849,13 @@
         <v>20</v>
       </c>
       <c r="B21" s="2">
-        <v>45971.510416666664</v>
+        <v>46331.427083333336</v>
+      </c>
+      <c r="C21" t="s">
+        <v>25</v>
+      </c>
+      <c r="D21" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
@@ -742,7 +863,10 @@
         <v>21</v>
       </c>
       <c r="B22" s="1">
-        <v>45974.552083333336</v>
+        <v>46338.427083333336</v>
+      </c>
+      <c r="C22" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
@@ -750,7 +874,13 @@
         <v>22</v>
       </c>
       <c r="B23" s="2">
-        <v>45978.510416666664</v>
+        <v>46343.59375</v>
+      </c>
+      <c r="C23" t="s">
+        <v>22</v>
+      </c>
+      <c r="D23" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
@@ -758,7 +888,13 @@
         <v>23</v>
       </c>
       <c r="B24" s="1">
-        <v>45981.552083333336</v>
+        <v>46345.427083333336</v>
+      </c>
+      <c r="C24" t="s">
+        <v>27</v>
+      </c>
+      <c r="D24" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
@@ -766,13 +902,10 @@
         <v>24</v>
       </c>
       <c r="B25" s="2">
-        <v>45985.510416666664</v>
+        <v>46350.59375</v>
       </c>
       <c r="C25" t="s">
-        <v>23</v>
-      </c>
-      <c r="D25" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
@@ -780,10 +913,10 @@
         <v>25</v>
       </c>
       <c r="B26" s="1">
-        <v>45988.552083333336</v>
+        <v>46352.427083333336</v>
       </c>
       <c r="C26" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
@@ -791,10 +924,10 @@
         <v>26</v>
       </c>
       <c r="B27" s="2">
-        <v>45992.510416666664</v>
+        <v>46357.59375</v>
       </c>
       <c r="C27" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
@@ -802,10 +935,10 @@
         <v>27</v>
       </c>
       <c r="B28" s="1">
-        <v>45995.552083333336</v>
+        <v>46359.427083333336</v>
       </c>
       <c r="C28" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
@@ -813,10 +946,10 @@
         <v>28</v>
       </c>
       <c r="B29" s="2">
-        <v>45999.510416666664</v>
+        <v>46364.59375</v>
       </c>
       <c r="C29" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
@@ -824,10 +957,10 @@
         <v>29</v>
       </c>
       <c r="B30" s="1">
-        <v>46002.552083333336</v>
+        <v>46366.427083333336</v>
       </c>
       <c r="C30" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
@@ -835,10 +968,10 @@
         <v>30</v>
       </c>
       <c r="B31" s="3">
-        <v>46006.510416666664</v>
+        <v>46371.59375</v>
       </c>
       <c r="C31" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ajout déclaration, exercices immer et usereducer
</commit_message>
<xml_diff>
--- a/template/horaire.xlsx
+++ b/template/horaire.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/etiennerivard/notes_de_cours/web3/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D8D34B2-5E2C-C346-A9F6-4A7443C01CEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32DC7004-F294-194A-8BDA-5BED8BA95A45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3000" yWindow="1580" windowWidth="25920" windowHeight="16440" xr2:uid="{4696F4E7-E751-AB46-8D30-A385E7EE1466}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="49">
   <si>
     <t>Date</t>
   </si>
@@ -177,6 +177,12 @@
   </si>
   <si>
     <t>[Typescript 2 et JavaScript asynchrone](exercices/typescript/typescript_async.md)</t>
+  </si>
+  <si>
+    <t>[React et useReducer](exercices/react/react_usereducer.md)</t>
+  </si>
+  <si>
+    <t>[Immer](exercices/outils/immer.md)</t>
   </si>
 </sst>
 </file>
@@ -701,6 +707,9 @@
       <c r="C9" t="s">
         <v>23</v>
       </c>
+      <c r="D9" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10">
@@ -711,6 +720,9 @@
       </c>
       <c r="C10" t="s">
         <v>24</v>
+      </c>
+      <c r="D10" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
correction horaire pour heure début jeudi
</commit_message>
<xml_diff>
--- a/template/horaire.xlsx
+++ b/template/horaire.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/etiennerivard/notes_de_cours/web3/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32DC7004-F294-194A-8BDA-5BED8BA95A45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04D6EA91-CC44-834A-955D-B1FBC3920AF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3000" yWindow="1580" windowWidth="25920" windowHeight="16440" xr2:uid="{4696F4E7-E751-AB46-8D30-A385E7EE1466}"/>
   </bookViews>
@@ -604,7 +604,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1">
-        <v>46254.427083333336</v>
+        <v>46254.34375</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -632,7 +632,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="1">
-        <v>46261.427083333336</v>
+        <v>46261.34375</v>
       </c>
       <c r="C4" t="s">
         <v>13</v>
@@ -646,7 +646,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="2">
-        <v>46268.427083333336</v>
+        <v>46268.34375</v>
       </c>
       <c r="C5" t="s">
         <v>15</v>
@@ -702,7 +702,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="2">
-        <v>46282.427083333336</v>
+        <v>46282.34375</v>
       </c>
       <c r="C9" t="s">
         <v>23</v>
@@ -730,7 +730,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="2">
-        <v>46289.427083333336</v>
+        <v>46289.34375</v>
       </c>
       <c r="C11" t="s">
         <v>11</v>
@@ -755,7 +755,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="2">
-        <v>46296.427083333336</v>
+        <v>46296.34375</v>
       </c>
       <c r="C13" t="s">
         <v>6</v>
@@ -780,7 +780,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="2">
-        <v>46303.427083333336</v>
+        <v>46303.34375</v>
       </c>
       <c r="C15" t="s">
         <v>5</v>
@@ -805,7 +805,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="2">
-        <v>46317.427083333336</v>
+        <v>46317.34375</v>
       </c>
       <c r="C17" t="s">
         <v>33</v>
@@ -833,7 +833,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="2">
-        <v>46324.427083333336</v>
+        <v>46324.34375</v>
       </c>
       <c r="C19" t="s">
         <v>32</v>
@@ -861,7 +861,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="2">
-        <v>46331.427083333336</v>
+        <v>46331.34375</v>
       </c>
       <c r="C21" t="s">
         <v>25</v>
@@ -875,7 +875,7 @@
         <v>21</v>
       </c>
       <c r="B22" s="1">
-        <v>46338.427083333336</v>
+        <v>46338.34375</v>
       </c>
       <c r="C22" t="s">
         <v>25</v>
@@ -900,7 +900,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="1">
-        <v>46345.427083333336</v>
+        <v>46345.34375</v>
       </c>
       <c r="C24" t="s">
         <v>27</v>
@@ -925,7 +925,7 @@
         <v>25</v>
       </c>
       <c r="B26" s="1">
-        <v>46352.427083333336</v>
+        <v>46352.34375</v>
       </c>
       <c r="C26" t="s">
         <v>16</v>
@@ -947,7 +947,7 @@
         <v>27</v>
       </c>
       <c r="B28" s="1">
-        <v>46359.427083333336</v>
+        <v>46359.34375</v>
       </c>
       <c r="C28" t="s">
         <v>16</v>
@@ -969,7 +969,7 @@
         <v>29</v>
       </c>
       <c r="B30" s="1">
-        <v>46366.427083333336</v>
+        <v>46366.34375</v>
       </c>
       <c r="C30" t="s">
         <v>17</v>

</xml_diff>

<commit_message>
ajout écran pour exercice intro next.js
</commit_message>
<xml_diff>
--- a/template/horaire.xlsx
+++ b/template/horaire.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/etiennerivard/notes_de_cours/web3/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04D6EA91-CC44-834A-955D-B1FBC3920AF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3857F36A-F138-FF4D-A592-EAD90C560C3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3000" yWindow="1580" windowWidth="25920" windowHeight="16440" xr2:uid="{4696F4E7-E751-AB46-8D30-A385E7EE1466}"/>
   </bookViews>
@@ -122,39 +122,12 @@
     <t>[Internationalisation avec Next.js](lecons/next.js/next_intl.md)</t>
   </si>
   <si>
-    <t>[Intro à Next.js](exercices/next_intro.md)</t>
-  </si>
-  <si>
-    <t>[Routage dans Next.js](exercices/next_routage.md)</t>
-  </si>
-  <si>
-    <t>[Composantes dans Next.js](exercices/next_composantes.md)</t>
-  </si>
-  <si>
-    <t>[Modes de rendu](exercices/next_modes_rendu.md)</t>
-  </si>
-  <si>
     <t>[Hydratation](lecons/next.js/hydratation.md)</t>
   </si>
   <si>
     <t xml:space="preserve">[Composantes serveur VS client](lecons/next.js/composantes.md) </t>
   </si>
   <si>
-    <t>[Hydratation](exercices/next_hydratation.md)</t>
-  </si>
-  <si>
-    <t>[Routes API](exercices/next_api_routes.md)</t>
-  </si>
-  <si>
-    <t>[ORM](exercices/next_orm.md)</t>
-  </si>
-  <si>
-    <t>[Server Actions](exercices/next_server_actions.md)</t>
-  </si>
-  <si>
-    <t>[Internationalisation](exercices/next_intl_exercice.md)</t>
-  </si>
-  <si>
     <t>[Introduction React](exercices/react/react_intro.md)</t>
   </si>
   <si>
@@ -183,6 +156,33 @@
   </si>
   <si>
     <t>[Immer](exercices/outils/immer.md)</t>
+  </si>
+  <si>
+    <t>[Intro à Next.js](exercices/nextjs/next_intro.md)</t>
+  </si>
+  <si>
+    <t>[Routage dans Next.js](exercices/nextjs/next_routage.md)</t>
+  </si>
+  <si>
+    <t>[Composantes dans Next.js](exercices/nextjs/next_composantes.md)</t>
+  </si>
+  <si>
+    <t>[Modes de rendu](exercices/nextjs/next_modes_rendu.md)</t>
+  </si>
+  <si>
+    <t>[Hydratation](exercices/nextjs/next_hydratation.md)</t>
+  </si>
+  <si>
+    <t>[Routes API](exercices/nextjs/next_api_routes.md)</t>
+  </si>
+  <si>
+    <t>[ORM](exercices/nextjs/next_orm.md)</t>
+  </si>
+  <si>
+    <t>[Server Actions](exercices/nextjs/next_server_actions.md)</t>
+  </si>
+  <si>
+    <t>[Internationalisation](exercices/nextjs/next_intl_exercice.md)</t>
   </si>
 </sst>
 </file>
@@ -610,7 +610,7 @@
         <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -624,7 +624,7 @@
         <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -638,7 +638,7 @@
         <v>13</v>
       </c>
       <c r="D4" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -652,7 +652,7 @@
         <v>15</v>
       </c>
       <c r="D5" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -666,7 +666,7 @@
         <v>14</v>
       </c>
       <c r="D6" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -680,7 +680,7 @@
         <v>10</v>
       </c>
       <c r="D7" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -694,7 +694,7 @@
         <v>26</v>
       </c>
       <c r="D8" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -708,7 +708,7 @@
         <v>23</v>
       </c>
       <c r="D9" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
@@ -722,7 +722,7 @@
         <v>24</v>
       </c>
       <c r="D10" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
@@ -736,7 +736,7 @@
         <v>11</v>
       </c>
       <c r="D11" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
@@ -772,7 +772,7 @@
         <v>7</v>
       </c>
       <c r="D14" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
@@ -797,7 +797,7 @@
         <v>19</v>
       </c>
       <c r="D16" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
@@ -808,10 +808,10 @@
         <v>46317.34375</v>
       </c>
       <c r="C17" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D17" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
@@ -825,7 +825,7 @@
         <v>20</v>
       </c>
       <c r="D18" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
@@ -836,10 +836,10 @@
         <v>46324.34375</v>
       </c>
       <c r="C19" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D19" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
@@ -853,7 +853,7 @@
         <v>21</v>
       </c>
       <c r="D20" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
@@ -867,7 +867,7 @@
         <v>25</v>
       </c>
       <c r="D21" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
@@ -892,7 +892,7 @@
         <v>22</v>
       </c>
       <c r="D23" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
@@ -906,7 +906,7 @@
         <v>27</v>
       </c>
       <c r="D24" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
correction leçon et exercice pour ORM
</commit_message>
<xml_diff>
--- a/template/horaire.xlsx
+++ b/template/horaire.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/etiennerivard/notes_de_cours/web3/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C82A622-F179-514F-854D-545DE187302C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19BDCBA9-49F5-D14C-B2E8-206DB0FC59BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3000" yWindow="1580" windowWidth="25920" windowHeight="16440" xr2:uid="{4696F4E7-E751-AB46-8D30-A385E7EE1466}"/>
   </bookViews>
@@ -850,10 +850,10 @@
         <v>46329.59375</v>
       </c>
       <c r="C20" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D20" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
@@ -866,9 +866,6 @@
       <c r="C21" t="s">
         <v>25</v>
       </c>
-      <c r="D21" t="s">
-        <v>45</v>
-      </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22">
@@ -878,7 +875,10 @@
         <v>46338.34375</v>
       </c>
       <c r="C22" t="s">
-        <v>25</v>
+        <v>21</v>
+      </c>
+      <c r="D22" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>